<commit_message>
Trixie treats sold loose: 100 g variants (PLU 00107-00111) + ArmSoft import 2026-10-15
Five Trixie dog treats (350/379/380/381/383) get a 100 g pack variant at the
bag rate +10% (user). ArmSoft: final/armsoft-2026-10-15 = yesterday's 22 new
goods + goods 0403/0516/0517/0552/0459 as weight goods (303 per kg, 003 bag).
Source of truth, 303 dog prices, scale/PLU files kept in step; the -100G SKU
counts as loose in check_codes and backfill-variant-codes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/final/Siruk-hx-303-prices-dog.xlsx
+++ b/final/Siruk-hx-303-prices-dog.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D74"/>
+  <dimension ref="A1:D79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1898,6 +1898,106 @@
         <v>8000</v>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Հյուրասիրություն շների Bony Mix` գունավոր ոսկորիկներ  կգ</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Soft Snack Bony Mix XXL — 1,800 g</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>00107</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Պեչենի շն.` գունավոր խառը ոսկորիկներ, մեծ կգ</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Cookie Bones — 1.3 kg</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>00108</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>4100</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Պեչենի շն.` գունավոր մանր կենդանիներ, Farmies   կգ</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Cookie Farmies — 1.3 kg</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>00109</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>4100</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Թխվածքաբլիթներ շն.` գառան մսով, կգ</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Cookie Giants with Lamb — 1.25 kg</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>00110</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>3700</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Պեչենի շն.` գունավոր օղակներ Vegan Loops,  կգ</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Cookie Snack Loops — 1.3 kg</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>00111</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>5100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Trixie 100 g loose: zoovet per-kg prices; ArmSoft split into new-goods and update-loose files
The 100 g variants now take zoovet.am's loose per-kg price / 10 (650/500/500/520/600),
price_source_url set. final/armsoft-2026-10-15: new-goods.xml + new-goods-prices.xlsx
(yesterday's 22 goods) and update-loose-goods.xml + update-loose-prices.xlsx (0403 0516
0517 0552 0459 as weight goods, 303 = 6500/5000/5000/5200/6000).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/final/Siruk-hx-303-prices-dog.xlsx
+++ b/final/Siruk-hx-303-prices-dog.xlsx
@@ -1915,7 +1915,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>7000</v>
+        <v>6500</v>
       </c>
     </row>
     <row r="76">
@@ -1935,7 +1935,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>4100</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="77">
@@ -1955,7 +1955,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>4100</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="78">
@@ -1975,7 +1975,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>3700</v>
+        <v>5200</v>
       </c>
     </row>
     <row r="79">
@@ -1995,7 +1995,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>5100</v>
+        <v>6000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Trixie 100 g loose: back to bag rate +10% (no rival sells them by 100 g)
zoovet.am sells all five only per 1 kg; the user's rule is a rival per-100 g
price or else our own. Site 700/410/410/370/510, price_source_url cleared;
ArmSoft 303 = 7000/4100/4100/3700/5100 in update-loose-prices.xlsx, final/ and
scale files in step.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/final/Siruk-hx-303-prices-dog.xlsx
+++ b/final/Siruk-hx-303-prices-dog.xlsx
@@ -1915,7 +1915,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>6500</v>
+        <v>7000</v>
       </c>
     </row>
     <row r="76">
@@ -1935,7 +1935,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>5000</v>
+        <v>4100</v>
       </c>
     </row>
     <row r="77">
@@ -1955,7 +1955,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>5000</v>
+        <v>4100</v>
       </c>
     </row>
     <row r="78">
@@ -1975,7 +1975,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>5200</v>
+        <v>3700</v>
       </c>
     </row>
     <row r="79">
@@ -1995,7 +1995,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>6000</v>
+        <v>5100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Trixie cookies 100 g: zoovet loose per-kg +10% (550/550/570/660); scale 5500/5500/5700/6600
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/final/Siruk-hx-303-prices-dog.xlsx
+++ b/final/Siruk-hx-303-prices-dog.xlsx
@@ -1935,7 +1935,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>4100</v>
+        <v>5500</v>
       </c>
     </row>
     <row r="77">
@@ -1955,7 +1955,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>4100</v>
+        <v>5500</v>
       </c>
     </row>
     <row r="78">
@@ -1975,7 +1975,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>3700</v>
+        <v>5700</v>
       </c>
     </row>
     <row r="79">
@@ -1995,7 +1995,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>5100</v>
+        <v>6600</v>
       </c>
     </row>
   </sheetData>

</xml_diff>